<commit_message>
penalty score table bug
</commit_message>
<xml_diff>
--- a/howell4x3.xlsx
+++ b/howell4x3.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Jul 30, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Aug 05, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 61</t>
+          <t>Name 89</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 83</t>
+          <t>Name 39</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 43</t>
+          <t>Name 77</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 43</t>
+          <t>Name 71</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 63</t>
+          <t>Name 34</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 45</t>
+          <t>Name 49</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 15</t>
+          <t>Name 45</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 70</t>
+          <t>Name 46</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -5572,15 +5572,15 @@
         <v/>
       </c>
       <c r="N4">
-        <f>K3-100</f>
+        <f>N3-100</f>
         <v/>
       </c>
       <c r="O4">
-        <f>L3-300</f>
+        <f>O3-300</f>
         <v/>
       </c>
       <c r="P4">
-        <f>L4*2</f>
+        <f>O4*2</f>
         <v/>
       </c>
     </row>
@@ -5622,15 +5622,15 @@
         <v/>
       </c>
       <c r="N5">
-        <f>K4-100</f>
+        <f>N4-100</f>
         <v/>
       </c>
       <c r="O5">
-        <f>L4-300</f>
+        <f>O4-300</f>
         <v/>
       </c>
       <c r="P5">
-        <f>L5*2</f>
+        <f>O5*2</f>
         <v/>
       </c>
     </row>
@@ -5672,15 +5672,15 @@
         <v/>
       </c>
       <c r="N6">
-        <f>K5-100</f>
+        <f>N5-100</f>
         <v/>
       </c>
       <c r="O6">
-        <f>L5-300</f>
+        <f>O5-300</f>
         <v/>
       </c>
       <c r="P6">
-        <f>L6*2</f>
+        <f>O6*2</f>
         <v/>
       </c>
     </row>
@@ -5722,15 +5722,15 @@
         <v/>
       </c>
       <c r="N7">
-        <f>K6-100</f>
+        <f>N6-100</f>
         <v/>
       </c>
       <c r="O7">
-        <f>L6-300</f>
+        <f>O6-300</f>
         <v/>
       </c>
       <c r="P7">
-        <f>L7*2</f>
+        <f>O7*2</f>
         <v/>
       </c>
     </row>
@@ -5772,15 +5772,15 @@
         <v/>
       </c>
       <c r="N8">
-        <f>K7-100</f>
+        <f>N7-100</f>
         <v/>
       </c>
       <c r="O8">
-        <f>L7-300</f>
+        <f>O7-300</f>
         <v/>
       </c>
       <c r="P8">
-        <f>L8*2</f>
+        <f>O8*2</f>
         <v/>
       </c>
     </row>
@@ -5822,15 +5822,15 @@
         <v/>
       </c>
       <c r="N9">
-        <f>K8-100</f>
+        <f>N8-100</f>
         <v/>
       </c>
       <c r="O9">
-        <f>L8-300</f>
+        <f>O8-300</f>
         <v/>
       </c>
       <c r="P9">
-        <f>L9*2</f>
+        <f>O9*2</f>
         <v/>
       </c>
     </row>
@@ -5877,15 +5877,15 @@
         <v/>
       </c>
       <c r="N10">
-        <f>K9-100</f>
+        <f>N9-100</f>
         <v/>
       </c>
       <c r="O10">
-        <f>L9-300</f>
+        <f>O9-300</f>
         <v/>
       </c>
       <c r="P10">
-        <f>L10*2</f>
+        <f>O10*2</f>
         <v/>
       </c>
     </row>
@@ -5927,15 +5927,15 @@
         <v/>
       </c>
       <c r="N11">
-        <f>K10-100</f>
+        <f>N10-100</f>
         <v/>
       </c>
       <c r="O11">
-        <f>L10-300</f>
+        <f>O10-300</f>
         <v/>
       </c>
       <c r="P11">
-        <f>L11*2</f>
+        <f>O11*2</f>
         <v/>
       </c>
     </row>
@@ -5977,15 +5977,15 @@
         <v/>
       </c>
       <c r="N12">
-        <f>K11-100</f>
+        <f>N11-100</f>
         <v/>
       </c>
       <c r="O12">
-        <f>L11-300</f>
+        <f>O11-300</f>
         <v/>
       </c>
       <c r="P12">
-        <f>L12*2</f>
+        <f>O12*2</f>
         <v/>
       </c>
     </row>
@@ -6027,15 +6027,15 @@
         <v/>
       </c>
       <c r="N13">
-        <f>K12-100</f>
+        <f>N12-100</f>
         <v/>
       </c>
       <c r="O13">
-        <f>L12-300</f>
+        <f>O12-300</f>
         <v/>
       </c>
       <c r="P13">
-        <f>L13*2</f>
+        <f>O13*2</f>
         <v/>
       </c>
     </row>
@@ -6077,15 +6077,15 @@
         <v/>
       </c>
       <c r="N14">
-        <f>K13-100</f>
+        <f>N13-100</f>
         <v/>
       </c>
       <c r="O14">
-        <f>L13-300</f>
+        <f>O13-300</f>
         <v/>
       </c>
       <c r="P14">
-        <f>L14*2</f>
+        <f>O14*2</f>
         <v/>
       </c>
     </row>
@@ -6127,15 +6127,15 @@
         <v/>
       </c>
       <c r="N15">
-        <f>K14-100</f>
+        <f>N14-100</f>
         <v/>
       </c>
       <c r="O15">
-        <f>L14-300</f>
+        <f>O14-300</f>
         <v/>
       </c>
       <c r="P15">
-        <f>L15*2</f>
+        <f>O15*2</f>
         <v/>
       </c>
     </row>

</xml_diff>